<commit_message>
agregue los arreglos de las skills
</commit_message>
<xml_diff>
--- a/Funcionalidades del Sistema Ferreteria.xlsx
+++ b/Funcionalidades del Sistema Ferreteria.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FerreteriaAldrete\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21AF10D5-D750-42A9-AB62-9CA7BB712120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2FBC41D-AE5D-428D-BF83-41E4EB42679C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="199">
   <si>
     <t>Actor</t>
   </si>
@@ -29967,14 +29967,18 @@
       <c r="A3" s="27" t="s">
         <v>158</v>
       </c>
-      <c r="B3" s="32"/>
+      <c r="B3" s="32" t="s">
+        <v>194</v>
+      </c>
       <c r="C3" s="27"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="27" t="s">
         <v>159</v>
       </c>
-      <c r="B4" s="27"/>
+      <c r="B4" s="32" t="s">
+        <v>194</v>
+      </c>
       <c r="C4" s="27"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>